<commit_message>
fix(applicants): align sample excel structure and keep users only in seed
</commit_message>
<xml_diff>
--- a/docs/06-data/import-data-sample.xlsx
+++ b/docs/06-data/import-data-sample.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="147" uniqueCount="120">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="213" uniqueCount="158">
   <si>
     <t>ลำดับ</t>
   </si>
@@ -157,27 +157,60 @@
     <t>หอพักที่ 26 มหาวิทยาลัยขอนแก่น (หอพักใน มข.)</t>
   </si>
   <si>
+    <t>950 บาท/เดือน (รวมค่าน้ำ-ไฟ)</t>
+  </si>
+  <si>
+    <t>4,500 บาท/เดือน</t>
+  </si>
+  <si>
+    <t>1,500 บาท/ภาคการศึกษา</t>
+  </si>
+  <si>
     <t>โน้ตบุ๊กและโทรศัพท์มือถือ</t>
   </si>
   <si>
     <t>รับจ้างทำแล็บคอมพิวเตอร์ 1,200 บาท/เดือน</t>
   </si>
   <si>
+    <t>52</t>
+  </si>
+  <si>
     <t>เกษตรกร (ทำไร่อ้อย)</t>
   </si>
   <si>
+    <t>8,000 บาท/เดือน</t>
+  </si>
+  <si>
     <t>มีชีวิตอยู่</t>
   </si>
   <si>
+    <t>49</t>
+  </si>
+  <si>
     <t>รับจ้างทั่วไป</t>
   </si>
   <si>
+    <t>6,500 บาท/เดือน</t>
+  </si>
+  <si>
     <t>อยู่ด้วยกัน</t>
   </si>
   <si>
     <t>บิดา-มารดา</t>
   </si>
   <si>
+    <t>บิดา</t>
+  </si>
+  <si>
+    <t>เกษตรกร</t>
+  </si>
+  <si>
+    <t>1</t>
+  </si>
+  <si>
+    <t>0</t>
+  </si>
+  <si>
     <t>กู้ยืม กยศ. ค่าเล่าเรียนและค่าครองชีพ</t>
   </si>
   <si>
@@ -187,7 +220,7 @@
     <t>https://www.google.com/maps?q=16.478950,102.825630</t>
   </si>
   <si>
-    <t>1409900123451</t>
+    <t>1409900123454</t>
   </si>
   <si>
     <t>653040015-8</t>
@@ -217,19 +250,37 @@
     <t>หอพักพิมานคอนโดปาร์ค กังสดาล มข. ต.ในเมือง อ.เมือง จ.ขอนแก่น</t>
   </si>
   <si>
+    <t>3,500 บาท/เดือน</t>
+  </si>
+  <si>
+    <t>5,000 บาท/เดือน</t>
+  </si>
+  <si>
+    <t>2,000 บาท/ภาคการศึกษา</t>
+  </si>
+  <si>
     <t>ไอแพดและโทรศัพท์มือถือ</t>
   </si>
   <si>
     <t>ไม่มีรายได้เสริม</t>
   </si>
   <si>
+    <t>56</t>
+  </si>
+  <si>
     <t>ค้าขายรายย่อย</t>
   </si>
   <si>
+    <t>9,000 บาท/เดือน</t>
+  </si>
+  <si>
+    <t>53</t>
+  </si>
+  <si>
     <t>แม่บ้าน</t>
   </si>
   <si>
-    <t>บิดา</t>
+    <t>2</t>
   </si>
   <si>
     <t>กู้ยืม กยศ.</t>
@@ -241,7 +292,7 @@
     <t>https://www.google.com/maps?q=16.463200,102.828100</t>
   </si>
   <si>
-    <t>1409900123460</t>
+    <t>1409900123462</t>
   </si>
   <si>
     <t>673040120-4</t>
@@ -268,18 +319,39 @@
     <t>หอพักศุภกฤต อพาร์ตเมนต์ หลังมอ ซอยวัดป่าโนนม่วง อ.เมือง จ.ขอนแก่น</t>
   </si>
   <si>
+    <t>2,800 บาท/เดือน</t>
+  </si>
+  <si>
+    <t>4,800 บาท/เดือน</t>
+  </si>
+  <si>
+    <t>1,800 บาท/ภาคการศึกษา</t>
+  </si>
+  <si>
     <t>แล็ปท็อปและสมาร์ตโฟน</t>
   </si>
   <si>
     <t>พนักงานร้านกาแฟพาร์ทไทม์ 2,000 บาท/เดือน</t>
   </si>
   <si>
+    <t>50</t>
+  </si>
+  <si>
     <t>รับจ้างขับรถส่งของ</t>
   </si>
   <si>
+    <t>11,000 บาท/เดือน</t>
+  </si>
+  <si>
+    <t>48</t>
+  </si>
+  <si>
     <t>พนักงานบริการ</t>
   </si>
   <si>
+    <t>8,500 บาท/เดือน</t>
+  </si>
+  <si>
     <t>หย่าร้าง</t>
   </si>
   <si>
@@ -292,7 +364,7 @@
     <t>https://www.google.com/maps?q=16.485120,102.816400</t>
   </si>
   <si>
-    <t>1409900123478</t>
+    <t>1409900123471</t>
   </si>
   <si>
     <t>643040210-9</t>
@@ -319,15 +391,33 @@
     <t>หอพักเจริญสุข ริมบึงหนองแวงตราชู กังสดาล ต.ในเมือง อ.เมือง จ.ขอนแก่น</t>
   </si>
   <si>
+    <t>3,200 บาท/เดือน</t>
+  </si>
+  <si>
+    <t>5,200 บาท/เดือน</t>
+  </si>
+  <si>
+    <t>1,200 บาท/ภาคการศึกษา</t>
+  </si>
+  <si>
     <t>คอมพิวเตอร์และโทรศัพท์มือถือ</t>
   </si>
   <si>
     <t>สอนพิเศษคณิตศาสตร์ 3,000 บาท/เดือน</t>
   </si>
   <si>
+    <t>58</t>
+  </si>
+  <si>
     <t>ข้าราชการบำนาญ</t>
   </si>
   <si>
+    <t>14,000 บาท/เดือน</t>
+  </si>
+  <si>
+    <t>55</t>
+  </si>
+  <si>
     <t>ค้าขาย</t>
   </si>
   <si>
@@ -337,7 +427,7 @@
     <t>https://www.google.com/maps?q=16.459500,102.831200</t>
   </si>
   <si>
-    <t>1409900123486</t>
+    <t>1409900123489</t>
   </si>
   <si>
     <t>663040332-1</t>
@@ -364,16 +454,40 @@
     <t>บ้านพักอาศัยส่วนตัว บ้านเลขที่ 124 หมู่ 3 ต.ศิลา อ.เมือง จ.ขอนแก่น</t>
   </si>
   <si>
+    <t>0 (บ้านพักตนเอง)</t>
+  </si>
+  <si>
+    <t>4,000 บาท/เดือน</t>
+  </si>
+  <si>
+    <t>1,000 บาท/ภาคการศึกษา</t>
+  </si>
+  <si>
     <t>โน้ตบุ๊ก</t>
   </si>
   <si>
+    <t>54</t>
+  </si>
+  <si>
     <t>ทำสวนและเกษตรกรรม</t>
   </si>
   <si>
+    <t>7,500 บาท/เดือน</t>
+  </si>
+  <si>
+    <t>51</t>
+  </si>
+  <si>
+    <t>เกษตรกรรม</t>
+  </si>
+  <si>
     <t>https://www.google.com/maps?q=16.498100,102.842500</t>
   </si>
   <si>
-    <t>1409900123494</t>
+    <t>1409900123497</t>
+  </si>
+  <si>
+    <t>*</t>
   </si>
 </sst>
 </file>
@@ -716,7 +830,7 @@
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
   </sheetPr>
-  <dimension ref="A1:AL7"/>
+  <dimension ref="A1:AS20"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0"/>
   <sheetData>
     <row r="1" spans="1:38" x14ac:dyDescent="0.25">
@@ -948,496 +1062,603 @@
         <v>36</v>
       </c>
     </row>
-    <row r="3" spans="2:37" x14ac:dyDescent="0.25">
-      <c r="B3">
+    <row r="3" spans="1:45" x14ac:dyDescent="0.25">
+      <c r="A3">
         <v>1</v>
       </c>
+      <c r="B3" t="s">
+        <v>37</v>
+      </c>
       <c r="C3" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="D3" t="s">
+        <v>39</v>
+      </c>
+      <c r="E3" t="s">
+        <v>40</v>
+      </c>
+      <c r="F3" t="s">
+        <v>41</v>
+      </c>
+      <c r="G3" t="s">
+        <v>42</v>
+      </c>
+      <c r="H3">
+        <v>2</v>
+      </c>
+      <c r="I3" t="s">
+        <v>43</v>
+      </c>
+      <c r="J3">
+        <v>3.25</v>
+      </c>
+      <c r="K3" t="s">
+        <v>44</v>
+      </c>
+      <c r="L3" t="s">
+        <v>45</v>
+      </c>
+      <c r="M3" t="s">
+        <v>46</v>
+      </c>
+      <c r="N3" t="s">
+        <v>47</v>
+      </c>
+      <c r="O3" t="s">
+        <v>48</v>
+      </c>
+      <c r="P3" t="s">
+        <v>49</v>
+      </c>
+      <c r="Q3" t="s">
+        <v>50</v>
+      </c>
+      <c r="R3" t="s">
+        <v>51</v>
+      </c>
+      <c r="S3" t="s">
+        <v>52</v>
+      </c>
+      <c r="T3" t="s">
+        <v>53</v>
+      </c>
+      <c r="U3" t="s">
+        <v>54</v>
+      </c>
+      <c r="V3" t="s">
+        <v>55</v>
+      </c>
+      <c r="W3" t="s">
+        <v>56</v>
+      </c>
+      <c r="X3" t="s">
+        <v>57</v>
+      </c>
+      <c r="Y3" t="s">
+        <v>58</v>
+      </c>
+      <c r="Z3" t="s">
+        <v>55</v>
+      </c>
+      <c r="AA3" t="s">
+        <v>59</v>
+      </c>
+      <c r="AB3" t="s">
+        <v>60</v>
+      </c>
+      <c r="AC3" t="s">
+        <v>61</v>
+      </c>
+      <c r="AD3" t="s">
+        <v>62</v>
+      </c>
+      <c r="AE3" t="s">
+        <v>54</v>
+      </c>
+      <c r="AF3" t="s">
+        <v>63</v>
+      </c>
+      <c r="AG3" t="s">
+        <v>64</v>
+      </c>
+      <c r="AH3" t="s">
+        <v>63</v>
+      </c>
+      <c r="AI3" t="s">
+        <v>65</v>
+      </c>
+      <c r="AJ3" t="s">
+        <v>66</v>
+      </c>
+      <c r="AK3" t="s">
+        <v>67</v>
+      </c>
+      <c r="AL3" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="4" spans="1:45" x14ac:dyDescent="0.25">
+      <c r="A4">
+        <v>2</v>
+      </c>
+      <c r="B4" t="s">
+        <v>69</v>
+      </c>
+      <c r="C4" t="s">
+        <v>70</v>
+      </c>
+      <c r="D4" t="s">
+        <v>71</v>
+      </c>
+      <c r="E4" t="s">
+        <v>72</v>
+      </c>
+      <c r="F4" t="s">
+        <v>41</v>
+      </c>
+      <c r="G4" t="s">
+        <v>73</v>
+      </c>
+      <c r="H4">
+        <v>3</v>
+      </c>
+      <c r="I4" t="s">
+        <v>74</v>
+      </c>
+      <c r="J4">
+        <v>2.85</v>
+      </c>
+      <c r="K4" t="s">
+        <v>75</v>
+      </c>
+      <c r="L4" t="s">
+        <v>76</v>
+      </c>
+      <c r="M4" t="s">
+        <v>77</v>
+      </c>
+      <c r="N4" t="s">
+        <v>78</v>
+      </c>
+      <c r="O4" t="s">
+        <v>79</v>
+      </c>
+      <c r="P4" t="s">
+        <v>80</v>
+      </c>
+      <c r="Q4" t="s">
+        <v>81</v>
+      </c>
+      <c r="R4" t="s">
+        <v>82</v>
+      </c>
+      <c r="S4" t="s">
+        <v>83</v>
+      </c>
+      <c r="T4" t="s">
+        <v>84</v>
+      </c>
+      <c r="U4" t="s">
+        <v>85</v>
+      </c>
+      <c r="V4" t="s">
+        <v>55</v>
+      </c>
+      <c r="W4" t="s">
+        <v>86</v>
+      </c>
+      <c r="X4" t="s">
+        <v>87</v>
+      </c>
+      <c r="Y4" t="s">
+        <v>64</v>
+      </c>
+      <c r="Z4" t="s">
+        <v>55</v>
+      </c>
+      <c r="AA4" t="s">
+        <v>59</v>
+      </c>
+      <c r="AB4" t="s">
+        <v>61</v>
+      </c>
+      <c r="AC4" t="s">
+        <v>61</v>
+      </c>
+      <c r="AD4" t="s">
+        <v>84</v>
+      </c>
+      <c r="AE4" t="s">
+        <v>85</v>
+      </c>
+      <c r="AF4" t="s">
+        <v>64</v>
+      </c>
+      <c r="AG4" t="s">
+        <v>64</v>
+      </c>
+      <c r="AH4" t="s">
+        <v>88</v>
+      </c>
+      <c r="AI4" t="s">
+        <v>89</v>
+      </c>
+      <c r="AJ4" t="s">
+        <v>90</v>
+      </c>
+      <c r="AK4" t="s">
+        <v>91</v>
+      </c>
+      <c r="AL4" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="5" spans="1:45" x14ac:dyDescent="0.25">
+      <c r="A5">
+        <v>3</v>
+      </c>
+      <c r="B5" t="s">
+        <v>93</v>
+      </c>
+      <c r="C5" t="s">
         <v>38</v>
       </c>
-      <c r="E3" t="s">
-        <v>39</v>
-      </c>
-      <c r="F3" t="s">
-        <v>40</v>
-      </c>
-      <c r="G3" t="s">
+      <c r="D5" t="s">
+        <v>94</v>
+      </c>
+      <c r="E5" t="s">
+        <v>95</v>
+      </c>
+      <c r="F5" t="s">
         <v>41</v>
       </c>
-      <c r="H3" t="s">
-        <v>42</v>
-      </c>
-      <c r="I3">
+      <c r="G5" t="s">
+        <v>96</v>
+      </c>
+      <c r="H5">
+        <v>1</v>
+      </c>
+      <c r="I5" t="s">
+        <v>97</v>
+      </c>
+      <c r="J5">
+        <v>3.4</v>
+      </c>
+      <c r="K5" t="s">
+        <v>98</v>
+      </c>
+      <c r="L5" t="s">
+        <v>99</v>
+      </c>
+      <c r="M5" t="s">
+        <v>100</v>
+      </c>
+      <c r="N5" t="s">
+        <v>101</v>
+      </c>
+      <c r="O5" t="s">
+        <v>102</v>
+      </c>
+      <c r="P5" t="s">
+        <v>103</v>
+      </c>
+      <c r="Q5" t="s">
+        <v>104</v>
+      </c>
+      <c r="R5" t="s">
+        <v>105</v>
+      </c>
+      <c r="S5" t="s">
+        <v>106</v>
+      </c>
+      <c r="T5" t="s">
+        <v>107</v>
+      </c>
+      <c r="U5" t="s">
+        <v>108</v>
+      </c>
+      <c r="V5" t="s">
+        <v>55</v>
+      </c>
+      <c r="W5" t="s">
+        <v>109</v>
+      </c>
+      <c r="X5" t="s">
+        <v>110</v>
+      </c>
+      <c r="Y5" t="s">
+        <v>111</v>
+      </c>
+      <c r="Z5" t="s">
+        <v>55</v>
+      </c>
+      <c r="AA5" t="s">
+        <v>112</v>
+      </c>
+      <c r="AB5" t="s">
+        <v>113</v>
+      </c>
+      <c r="AC5" t="s">
+        <v>113</v>
+      </c>
+      <c r="AD5" t="s">
+        <v>110</v>
+      </c>
+      <c r="AE5" t="s">
+        <v>111</v>
+      </c>
+      <c r="AF5" t="s">
+        <v>64</v>
+      </c>
+      <c r="AG5" t="s">
+        <v>63</v>
+      </c>
+      <c r="AH5" t="s">
+        <v>63</v>
+      </c>
+      <c r="AI5" t="s">
+        <v>114</v>
+      </c>
+      <c r="AJ5" t="s">
+        <v>66</v>
+      </c>
+      <c r="AK5" t="s">
+        <v>115</v>
+      </c>
+      <c r="AL5" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="6" spans="1:45" x14ac:dyDescent="0.25">
+      <c r="A6">
+        <v>4</v>
+      </c>
+      <c r="B6" t="s">
+        <v>117</v>
+      </c>
+      <c r="C6" t="s">
+        <v>70</v>
+      </c>
+      <c r="D6" t="s">
+        <v>118</v>
+      </c>
+      <c r="E6" t="s">
+        <v>119</v>
+      </c>
+      <c r="F6" t="s">
+        <v>41</v>
+      </c>
+      <c r="G6" t="s">
+        <v>120</v>
+      </c>
+      <c r="H6">
+        <v>4</v>
+      </c>
+      <c r="I6" t="s">
+        <v>121</v>
+      </c>
+      <c r="J6">
+        <v>3.12</v>
+      </c>
+      <c r="K6" t="s">
+        <v>122</v>
+      </c>
+      <c r="L6" t="s">
+        <v>123</v>
+      </c>
+      <c r="M6" t="s">
+        <v>124</v>
+      </c>
+      <c r="N6" t="s">
+        <v>125</v>
+      </c>
+      <c r="O6" t="s">
+        <v>126</v>
+      </c>
+      <c r="P6" t="s">
+        <v>127</v>
+      </c>
+      <c r="Q6" t="s">
+        <v>128</v>
+      </c>
+      <c r="R6" t="s">
+        <v>129</v>
+      </c>
+      <c r="S6" t="s">
+        <v>130</v>
+      </c>
+      <c r="T6" t="s">
+        <v>131</v>
+      </c>
+      <c r="U6" t="s">
+        <v>132</v>
+      </c>
+      <c r="V6" t="s">
+        <v>55</v>
+      </c>
+      <c r="W6" t="s">
+        <v>133</v>
+      </c>
+      <c r="X6" t="s">
+        <v>134</v>
+      </c>
+      <c r="Y6" t="s">
+        <v>85</v>
+      </c>
+      <c r="Z6" t="s">
+        <v>55</v>
+      </c>
+      <c r="AA6" t="s">
+        <v>59</v>
+      </c>
+      <c r="AB6" t="s">
+        <v>60</v>
+      </c>
+      <c r="AC6" t="s">
+        <v>61</v>
+      </c>
+      <c r="AD6" t="s">
+        <v>131</v>
+      </c>
+      <c r="AE6" t="s">
+        <v>132</v>
+      </c>
+      <c r="AF6" t="s">
+        <v>63</v>
+      </c>
+      <c r="AG6" t="s">
+        <v>64</v>
+      </c>
+      <c r="AH6" t="s">
+        <v>64</v>
+      </c>
+      <c r="AI6" t="s">
+        <v>89</v>
+      </c>
+      <c r="AJ6" t="s">
+        <v>135</v>
+      </c>
+      <c r="AK6" t="s">
+        <v>136</v>
+      </c>
+      <c r="AL6" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="7" spans="1:45" x14ac:dyDescent="0.25">
+      <c r="A7">
+        <v>5</v>
+      </c>
+      <c r="B7" t="s">
+        <v>138</v>
+      </c>
+      <c r="C7" t="s">
+        <v>38</v>
+      </c>
+      <c r="D7" t="s">
+        <v>139</v>
+      </c>
+      <c r="E7" t="s">
+        <v>140</v>
+      </c>
+      <c r="F7" t="s">
+        <v>41</v>
+      </c>
+      <c r="G7" t="s">
+        <v>141</v>
+      </c>
+      <c r="H7">
         <v>2</v>
       </c>
-      <c r="J3" t="s">
-        <v>43</v>
-      </c>
-      <c r="K3">
-        <v>3.25</v>
-      </c>
-      <c r="L3" t="s">
-        <v>44</v>
-      </c>
-      <c r="M3" t="s">
-        <v>45</v>
-      </c>
-      <c r="N3" t="s">
-        <v>46</v>
-      </c>
-      <c r="O3">
-        <v>950</v>
-      </c>
-      <c r="P3">
-        <v>4500</v>
-      </c>
-      <c r="Q3">
-        <v>1500</v>
-      </c>
-      <c r="R3" t="s">
-        <v>47</v>
-      </c>
-      <c r="S3" t="s">
-        <v>48</v>
-      </c>
-      <c r="T3">
-        <v>52</v>
-      </c>
-      <c r="U3" t="s">
-        <v>49</v>
-      </c>
-      <c r="V3">
-        <v>8000</v>
-      </c>
-      <c r="W3" t="s">
-        <v>50</v>
-      </c>
-      <c r="X3">
-        <v>49</v>
-      </c>
-      <c r="Y3" t="s">
-        <v>51</v>
-      </c>
-      <c r="Z3">
-        <v>6500</v>
-      </c>
-      <c r="AA3" t="s">
-        <v>50</v>
-      </c>
-      <c r="AB3" t="s">
-        <v>52</v>
-      </c>
-      <c r="AC3" t="s">
-        <v>53</v>
-      </c>
-      <c r="AH3" t="s">
-        <v>54</v>
-      </c>
-      <c r="AI3" t="s">
+      <c r="I7" t="s">
+        <v>142</v>
+      </c>
+      <c r="J7">
+        <v>2.95</v>
+      </c>
+      <c r="K7" t="s">
+        <v>143</v>
+      </c>
+      <c r="L7" t="s">
+        <v>144</v>
+      </c>
+      <c r="M7" t="s">
+        <v>145</v>
+      </c>
+      <c r="N7" t="s">
+        <v>146</v>
+      </c>
+      <c r="O7" t="s">
+        <v>147</v>
+      </c>
+      <c r="P7" t="s">
+        <v>148</v>
+      </c>
+      <c r="Q7" t="s">
+        <v>149</v>
+      </c>
+      <c r="R7" t="s">
+        <v>82</v>
+      </c>
+      <c r="S7" t="s">
+        <v>150</v>
+      </c>
+      <c r="T7" t="s">
+        <v>151</v>
+      </c>
+      <c r="U7" t="s">
+        <v>152</v>
+      </c>
+      <c r="V7" t="s">
         <v>55</v>
       </c>
-      <c r="AJ3" t="s">
-        <v>56</v>
-      </c>
-      <c r="AK3" t="s">
-        <v>57</v>
+      <c r="W7" t="s">
+        <v>153</v>
+      </c>
+      <c r="X7" t="s">
+        <v>87</v>
+      </c>
+      <c r="Y7" t="s">
+        <v>64</v>
+      </c>
+      <c r="Z7" t="s">
+        <v>55</v>
+      </c>
+      <c r="AA7" t="s">
+        <v>59</v>
+      </c>
+      <c r="AB7" t="s">
+        <v>61</v>
+      </c>
+      <c r="AC7" t="s">
+        <v>61</v>
+      </c>
+      <c r="AD7" t="s">
+        <v>154</v>
+      </c>
+      <c r="AE7" t="s">
+        <v>152</v>
+      </c>
+      <c r="AF7" t="s">
+        <v>64</v>
+      </c>
+      <c r="AG7" t="s">
+        <v>64</v>
+      </c>
+      <c r="AH7" t="s">
+        <v>88</v>
+      </c>
+      <c r="AI7" t="s">
+        <v>89</v>
+      </c>
+      <c r="AJ7" t="s">
+        <v>66</v>
+      </c>
+      <c r="AK7" t="s">
+        <v>155</v>
+      </c>
+      <c r="AL7" t="s">
+        <v>156</v>
       </c>
     </row>
-    <row r="4" spans="2:37" x14ac:dyDescent="0.25">
-      <c r="B4">
-        <v>2</v>
-      </c>
-      <c r="C4" t="s">
-        <v>58</v>
-      </c>
-      <c r="D4" t="s">
-        <v>59</v>
-      </c>
-      <c r="E4" t="s">
-        <v>60</v>
-      </c>
-      <c r="F4" t="s">
-        <v>61</v>
-      </c>
-      <c r="G4" t="s">
-        <v>41</v>
-      </c>
-      <c r="H4" t="s">
-        <v>62</v>
-      </c>
-      <c r="I4">
-        <v>3</v>
-      </c>
-      <c r="J4" t="s">
-        <v>63</v>
-      </c>
-      <c r="K4">
-        <v>2.85</v>
-      </c>
-      <c r="L4" t="s">
-        <v>64</v>
-      </c>
-      <c r="M4" t="s">
-        <v>65</v>
-      </c>
-      <c r="N4" t="s">
-        <v>66</v>
-      </c>
-      <c r="O4">
-        <v>3500</v>
-      </c>
-      <c r="P4">
-        <v>5000</v>
-      </c>
-      <c r="Q4">
-        <v>2000</v>
-      </c>
-      <c r="R4" t="s">
-        <v>67</v>
-      </c>
-      <c r="S4" t="s">
-        <v>68</v>
-      </c>
-      <c r="T4">
-        <v>56</v>
-      </c>
-      <c r="U4" t="s">
-        <v>69</v>
-      </c>
-      <c r="V4">
-        <v>9000</v>
-      </c>
-      <c r="W4" t="s">
-        <v>50</v>
-      </c>
-      <c r="X4">
-        <v>53</v>
-      </c>
-      <c r="Y4" t="s">
-        <v>70</v>
-      </c>
-      <c r="Z4">
-        <v>0</v>
-      </c>
-      <c r="AA4" t="s">
-        <v>50</v>
-      </c>
-      <c r="AB4" t="s">
-        <v>52</v>
-      </c>
-      <c r="AC4" t="s">
-        <v>71</v>
-      </c>
-      <c r="AH4" t="s">
-        <v>72</v>
-      </c>
-      <c r="AI4" t="s">
-        <v>73</v>
-      </c>
-      <c r="AJ4" t="s">
-        <v>74</v>
-      </c>
-      <c r="AK4" t="s">
-        <v>75</v>
+    <row r="8" spans="1:45" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>157</v>
       </c>
     </row>
-    <row r="5" spans="2:37" x14ac:dyDescent="0.25">
-      <c r="B5">
-        <v>3</v>
-      </c>
-      <c r="C5" t="s">
-        <v>76</v>
-      </c>
-      <c r="D5" t="s">
-        <v>38</v>
-      </c>
-      <c r="E5" t="s">
-        <v>77</v>
-      </c>
-      <c r="F5" t="s">
-        <v>78</v>
-      </c>
-      <c r="G5" t="s">
-        <v>41</v>
-      </c>
-      <c r="H5" t="s">
-        <v>79</v>
-      </c>
-      <c r="I5">
-        <v>1</v>
-      </c>
-      <c r="J5" t="s">
-        <v>80</v>
-      </c>
-      <c r="K5">
-        <v>3.4</v>
-      </c>
-      <c r="L5" t="s">
-        <v>81</v>
-      </c>
-      <c r="M5" t="s">
-        <v>82</v>
-      </c>
-      <c r="N5" t="s">
-        <v>83</v>
-      </c>
-      <c r="O5">
-        <v>2800</v>
-      </c>
-      <c r="P5">
-        <v>4800</v>
-      </c>
-      <c r="Q5">
-        <v>1800</v>
-      </c>
-      <c r="R5" t="s">
-        <v>84</v>
-      </c>
-      <c r="S5" t="s">
-        <v>85</v>
-      </c>
-      <c r="T5">
-        <v>50</v>
-      </c>
-      <c r="U5" t="s">
-        <v>86</v>
-      </c>
-      <c r="V5">
-        <v>11000</v>
-      </c>
-      <c r="W5" t="s">
-        <v>50</v>
-      </c>
-      <c r="X5">
-        <v>48</v>
-      </c>
-      <c r="Y5" t="s">
-        <v>87</v>
-      </c>
-      <c r="Z5">
-        <v>8500</v>
-      </c>
-      <c r="AA5" t="s">
-        <v>50</v>
-      </c>
-      <c r="AB5" t="s">
-        <v>88</v>
-      </c>
-      <c r="AC5" t="s">
-        <v>89</v>
-      </c>
-      <c r="AH5" t="s">
-        <v>90</v>
-      </c>
-      <c r="AI5" t="s">
-        <v>55</v>
-      </c>
-      <c r="AJ5" t="s">
-        <v>91</v>
-      </c>
-      <c r="AK5" t="s">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="6" spans="2:37" x14ac:dyDescent="0.25">
-      <c r="B6">
-        <v>4</v>
-      </c>
-      <c r="C6" t="s">
-        <v>93</v>
-      </c>
-      <c r="D6" t="s">
-        <v>59</v>
-      </c>
-      <c r="E6" t="s">
-        <v>94</v>
-      </c>
-      <c r="F6" t="s">
-        <v>95</v>
-      </c>
-      <c r="G6" t="s">
-        <v>41</v>
-      </c>
-      <c r="H6" t="s">
-        <v>96</v>
-      </c>
-      <c r="I6">
-        <v>4</v>
-      </c>
-      <c r="J6" t="s">
-        <v>97</v>
-      </c>
-      <c r="K6">
-        <v>3.12</v>
-      </c>
-      <c r="L6" t="s">
-        <v>98</v>
-      </c>
-      <c r="M6" t="s">
-        <v>99</v>
-      </c>
-      <c r="N6" t="s">
-        <v>100</v>
-      </c>
-      <c r="O6">
-        <v>3200</v>
-      </c>
-      <c r="P6">
-        <v>5200</v>
-      </c>
-      <c r="Q6">
-        <v>1200</v>
-      </c>
-      <c r="R6" t="s">
-        <v>101</v>
-      </c>
-      <c r="S6" t="s">
-        <v>102</v>
-      </c>
-      <c r="T6">
-        <v>58</v>
-      </c>
-      <c r="U6" t="s">
-        <v>103</v>
-      </c>
-      <c r="V6">
-        <v>14000</v>
-      </c>
-      <c r="W6" t="s">
-        <v>50</v>
-      </c>
-      <c r="X6">
-        <v>55</v>
-      </c>
-      <c r="Y6" t="s">
-        <v>104</v>
-      </c>
-      <c r="Z6">
-        <v>9000</v>
-      </c>
-      <c r="AA6" t="s">
-        <v>50</v>
-      </c>
-      <c r="AB6" t="s">
-        <v>52</v>
-      </c>
-      <c r="AC6" t="s">
-        <v>53</v>
-      </c>
-      <c r="AH6" t="s">
-        <v>72</v>
-      </c>
-      <c r="AI6" t="s">
-        <v>105</v>
-      </c>
-      <c r="AJ6" t="s">
-        <v>106</v>
-      </c>
-      <c r="AK6" t="s">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="7" spans="2:37" x14ac:dyDescent="0.25">
-      <c r="B7">
-        <v>5</v>
-      </c>
-      <c r="C7" t="s">
-        <v>108</v>
-      </c>
-      <c r="D7" t="s">
-        <v>38</v>
-      </c>
-      <c r="E7" t="s">
-        <v>109</v>
-      </c>
-      <c r="F7" t="s">
-        <v>110</v>
-      </c>
-      <c r="G7" t="s">
-        <v>41</v>
-      </c>
-      <c r="H7" t="s">
-        <v>111</v>
-      </c>
-      <c r="I7">
-        <v>2</v>
-      </c>
-      <c r="J7" t="s">
-        <v>112</v>
-      </c>
-      <c r="K7">
-        <v>2.95</v>
-      </c>
-      <c r="L7" t="s">
-        <v>113</v>
-      </c>
-      <c r="M7" t="s">
-        <v>114</v>
-      </c>
-      <c r="N7" t="s">
-        <v>115</v>
-      </c>
-      <c r="O7">
-        <v>0</v>
-      </c>
-      <c r="P7">
-        <v>4000</v>
-      </c>
-      <c r="Q7">
-        <v>1000</v>
-      </c>
-      <c r="R7" t="s">
-        <v>116</v>
-      </c>
-      <c r="S7" t="s">
-        <v>68</v>
-      </c>
-      <c r="T7">
-        <v>54</v>
-      </c>
-      <c r="U7" t="s">
-        <v>117</v>
-      </c>
-      <c r="V7">
-        <v>7500</v>
-      </c>
-      <c r="W7" t="s">
-        <v>50</v>
-      </c>
-      <c r="X7">
-        <v>51</v>
-      </c>
-      <c r="Y7" t="s">
-        <v>70</v>
-      </c>
-      <c r="Z7">
-        <v>0</v>
-      </c>
-      <c r="AA7" t="s">
-        <v>50</v>
-      </c>
-      <c r="AB7" t="s">
-        <v>52</v>
-      </c>
-      <c r="AC7" t="s">
-        <v>71</v>
-      </c>
-      <c r="AH7" t="s">
-        <v>72</v>
-      </c>
-      <c r="AI7" t="s">
-        <v>55</v>
-      </c>
-      <c r="AJ7" t="s">
-        <v>118</v>
-      </c>
-      <c r="AK7" t="s">
-        <v>119</v>
-      </c>
-    </row>
+    <row r="9" spans="1:45" x14ac:dyDescent="0.25"/>
+    <row r="10" spans="1:45" x14ac:dyDescent="0.25"/>
+    <row r="11" spans="1:45" x14ac:dyDescent="0.25"/>
+    <row r="12" spans="1:45" x14ac:dyDescent="0.25"/>
+    <row r="13" spans="1:45" x14ac:dyDescent="0.25"/>
+    <row r="14" spans="1:45" x14ac:dyDescent="0.25"/>
+    <row r="15" spans="1:45" x14ac:dyDescent="0.25"/>
+    <row r="16" spans="1:45" x14ac:dyDescent="0.25"/>
+    <row r="17" spans="1:45" x14ac:dyDescent="0.25"/>
+    <row r="18" spans="1:45" x14ac:dyDescent="0.25"/>
+    <row r="19" spans="1:45" x14ac:dyDescent="0.25"/>
+    <row r="20" spans="1:45" x14ac:dyDescent="0.25"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>